<commit_message>
Update NG Swing GDD v2 master prices
</commit_message>
<xml_diff>
--- a/master/master_ng_swing_gdd_v2.xlsx
+++ b/master/master_ng_swing_gdd_v2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="NG Swing GDD" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NG Swing GDD'!$A$1:$BR$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NG Swing GDD'!$A$1:$BR$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BR3"/>
+  <dimension ref="A1:BR5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1303,8 +1303,436 @@
         <v>-1.75</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>2.165</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>2.245</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>2.425</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>2.735</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>3.215</v>
+      </c>
+      <c r="R4" s="3" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="S4" s="3" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="T4" s="3" t="n">
+        <v>2.745</v>
+      </c>
+      <c r="U4" s="3" t="n">
+        <v>2.375</v>
+      </c>
+      <c r="V4" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="W4" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="X4" s="3" t="n">
+        <v>2.665</v>
+      </c>
+      <c r="Y4" s="3" t="n">
+        <v>2.715</v>
+      </c>
+      <c r="Z4" s="3" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="AA4" s="3" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="AB4" s="3" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="AC4" s="3" t="n">
+        <v>2.245</v>
+      </c>
+      <c r="AD4" s="3" t="n">
+        <v>1.245</v>
+      </c>
+      <c r="AE4" s="3" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="AF4" s="3" t="n">
+        <v>2.075</v>
+      </c>
+      <c r="AG4" s="3" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="AH4" s="3" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="AI4" s="3" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="AJ4" s="3" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="AK4" s="3" t="n">
+        <v>2.725</v>
+      </c>
+      <c r="AL4" s="3" t="n">
+        <v>2.255</v>
+      </c>
+      <c r="AM4" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="AN4" s="3" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="AO4" s="3" t="n">
+        <v>4.315</v>
+      </c>
+      <c r="AP4" s="3" t="n">
+        <v>2.615</v>
+      </c>
+      <c r="AQ4" s="3" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="AR4" s="3" t="n">
+        <v>2.915</v>
+      </c>
+      <c r="AS4" s="3" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="AT4" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AU4" s="3" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="AV4" s="3" t="n">
+        <v>2.905</v>
+      </c>
+      <c r="AW4" s="3" t="n">
+        <v>4.295</v>
+      </c>
+      <c r="AX4" s="3" t="n">
+        <v>2.795</v>
+      </c>
+      <c r="AY4" s="3" t="n">
+        <v>2.715</v>
+      </c>
+      <c r="AZ4" s="3" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="BA4" s="3" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="BB4" s="3" t="n">
+        <v>2.405</v>
+      </c>
+      <c r="BC4" s="3" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="BD4" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="BE4" s="3" t="n">
+        <v>2.825</v>
+      </c>
+      <c r="BF4" s="3" t="n">
+        <v>2.525</v>
+      </c>
+      <c r="BG4" s="3" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="BH4" s="3" t="n">
+        <v>2.835</v>
+      </c>
+      <c r="BI4" s="3" t="n">
+        <v>4.275</v>
+      </c>
+      <c r="BJ4" s="3" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="BK4" s="3" t="n">
+        <v>2.485</v>
+      </c>
+      <c r="BL4" s="3" t="n">
+        <v>3.555</v>
+      </c>
+      <c r="BM4" s="3" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="BN4" s="3" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="BO4" s="3" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="BP4" s="3" t="n">
+        <v>2.525</v>
+      </c>
+      <c r="BQ4" s="3" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="BR4" s="3" t="n">
+        <v>1.495</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>2.615</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>2.975</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>2.815</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>2.815</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>1.935</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>1.775</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>2.765</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>3.285</v>
+      </c>
+      <c r="R5" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="S5" s="3" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="T5" s="3" t="n">
+        <v>2.795</v>
+      </c>
+      <c r="U5" s="3" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="V5" s="3" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="W5" s="3" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="X5" s="3" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="Y5" s="3" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="Z5" s="3" t="n">
+        <v>2.755</v>
+      </c>
+      <c r="AA5" s="3" t="n">
+        <v>2.665</v>
+      </c>
+      <c r="AB5" s="3" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="AC5" s="3" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="AD5" s="3" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="AE5" s="3" t="n">
+        <v>2.655</v>
+      </c>
+      <c r="AF5" s="3" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="AG5" s="3" t="n">
+        <v>1.315</v>
+      </c>
+      <c r="AH5" s="3" t="n">
+        <v>2.635</v>
+      </c>
+      <c r="AI5" s="3" t="n">
+        <v>1.775</v>
+      </c>
+      <c r="AJ5" s="3" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="AK5" s="3" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="AL5" s="3" t="n">
+        <v>2.005</v>
+      </c>
+      <c r="AM5" s="3" t="n">
+        <v>2.535</v>
+      </c>
+      <c r="AN5" s="3" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="AO5" s="3" t="n">
+        <v>4.415</v>
+      </c>
+      <c r="AP5" s="3" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="AQ5" s="3" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="AR5" s="3" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="AS5" s="3" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="AT5" s="3" t="n">
+        <v>2.495</v>
+      </c>
+      <c r="AU5" s="3" t="n">
+        <v>2.775</v>
+      </c>
+      <c r="AV5" s="3" t="n">
+        <v>2.975</v>
+      </c>
+      <c r="AW5" s="3" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="AX5" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="AY5" s="3" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="AZ5" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="BA5" s="3" t="n">
+        <v>2.515</v>
+      </c>
+      <c r="BB5" s="3" t="n">
+        <v>2.375</v>
+      </c>
+      <c r="BC5" s="3" t="n">
+        <v>2.965</v>
+      </c>
+      <c r="BD5" s="3" t="n">
+        <v>2.785</v>
+      </c>
+      <c r="BE5" s="3" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="BF5" s="3" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="BG5" s="3" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="BH5" s="3" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="BI5" s="3" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="BJ5" s="3" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="BK5" s="3" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="BL5" s="3" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="BM5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="BN5" s="3" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="BO5" s="3" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="BP5" s="3" t="n">
+        <v>2.515</v>
+      </c>
+      <c r="BQ5" s="3" t="n">
+        <v>2.825</v>
+      </c>
+      <c r="BR5" s="3" t="n">
+        <v>1.805</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:BR3"/>
+  <autoFilter ref="A1:BR5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>